<commit_message>
# 2) git add tests/factories.py tests/test_invoice_service.py test: cover invoice and import-rule services
- Update test_invoice_service to the current API: confirmed/paid booleans
  (no VoucherStatus), split confirm_invoice/register_payment, and
  InvoiceConfirmationError from exceptions.
- Fix factories for new NOT NULL columns (condicion_iva, doc_type,
  iva_aliquot); add make_category and make_import_rule.
- Add resolve_rule_for_classification tests: no-match->create,
  ecc-match->reuse, conflict->raise, force->update.
</commit_message>
<xml_diff>
--- a/Planilla de Flujo 2026-01.xlsx
+++ b/Planilla de Flujo 2026-01.xlsx
@@ -12800,7 +12800,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1156611.23</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -12821,7 +12821,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>163000</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -12842,7 +12842,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -12863,7 +12863,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>373000</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -12884,7 +12884,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>63399.09</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -12905,7 +12905,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>27483.75</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -12947,7 +12947,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>461000</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -12968,7 +12968,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>139815.62</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>137381.47</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -13010,7 +13010,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>117681.67</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -13031,7 +13031,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>17414.72</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -13052,7 +13052,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -13094,7 +13094,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>191000</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -13115,7 +13115,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -13157,7 +13157,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>119787.4</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -13178,7 +13178,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>191000</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -13220,7 +13220,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>8949.059999999999</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -13284,7 +13284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13314,6 +13314,762 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="67" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AYSA Venezuela $ 68,461.96 VISA</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>68461.96000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="67" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AYSA Aroma $15.800 VISA</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>15800</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="67" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Metrogas 5/12 $ 7,960.65 VISA</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7960.65</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="67" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Metrogas Aroma $ 38,758.28 VISA</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>38758.28</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Movistar Aroma $ 25.883.75 VISA</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>25883.75</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Movistar Todos $59.554.98 VISA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>59554.98</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Telecentro Tia  $ 46,679.87 VISA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>46679.87</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Metrogas Tia $9196.59 VISA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9196.59</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Metrogas 6/12 $7960.65 VISA</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7960.65</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Metrogas Aroma $ 38,835.75 VISA</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>38835.75</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="67" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AYSA Aroma $16285.86 VISA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>16285.86</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="67" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AYSA Venezuela   $70565.34 VISA</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>70565.34</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="67" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Telecentro Tia  $ 47979.87 VISA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>47979.87</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="67" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Metrogas Tia $8366.82 VISA</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8366.82</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="67" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Metrogas Aroma $36462.09 VISA</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>36462.09</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="67" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Metrogas 7/12 $7,960.65 VISA</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>7960.65</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="67" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AYSA Venezuela $ 75,456.52 VISA</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>75456.52</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="67" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Movistar Aroma $29752.50 VISA</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>29752.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Movistar Todos $66670.66 VISA</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>66670.66</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="67" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Telecentro TIA $ 56793 VISA</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>56793</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="67" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Metrogas TIA $8426.21 VISA</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>8426.209999999999</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="67" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Metrogas Aroma $36,585.19 VISA</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>36585.19</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="67" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Metrogas 8/12 $7960.65 VISA</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>7960.65</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="67" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Metrogas v.gomez $37528.68 VISA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>37528.68</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="67" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Movistar Todos $ 67352.34 VISA</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>67352.34</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="67" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Movistar  Aroma $31900 VISA</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>31900</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="67" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Telecentro TIA $56793 VISA</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>56793</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="67" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Metrogas TIA $ 8.952,93 VISA</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>8952.93</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="67" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Metrogas V.gomez $37202.35 VISA</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>37202.35</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="67" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Metrogas Aroma $ 45,445.01 VISA</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>45445.01</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Metrogas 9/12 VISA $7960.65</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>7960.65</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="67" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>AYSA Aroma $ 18,319.38 VISA</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>18319.38</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="67" t="n">
+        <v>45784</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Movistar ARoma $34123.75 VISA</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>34123.75</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="67" t="n">
+        <v>45784</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Movistar Todos $70.771.44 VISA</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>70771.44</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>AYSA Venezuela $ 79,376.39 VISA</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>79376.39</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="67" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Telecentro TIA $56793 VISA</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>56793</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>